<commit_message>
Updated Fixes For POM Modules
Updated Fixes For POM Modules
</commit_message>
<xml_diff>
--- a/testdata/DirectGrn.xlsx
+++ b/testdata/DirectGrn.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2772" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="264">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -289,10 +289,10 @@
     <t>INS WH-1</t>
   </si>
   <si>
-    <t>1432</t>
+    <t>1492</t>
   </si>
   <si>
-    <t>5315.99665</t>
+    <t>5277.91012</t>
   </si>
   <si>
     <t>Receipt Qty &amp; Unit cost</t>
@@ -328,10 +328,10 @@
     <t>4</t>
   </si>
   <si>
-    <t>426</t>
+    <t>454</t>
   </si>
   <si>
-    <t>6694.90186</t>
+    <t>6732.74603</t>
   </si>
   <si>
     <t>82.12</t>
@@ -352,10 +352,10 @@
     <t>3</t>
   </si>
   <si>
-    <t>1392</t>
+    <t>1512</t>
   </si>
   <si>
-    <t>3604.92118</t>
+    <t>3626.96254</t>
   </si>
   <si>
     <t>43.3</t>
@@ -727,13 +727,115 @@
     <t>GWL_Item_FP_Pl_Dissimilar_01</t>
   </si>
   <si>
+    <t>12978.9</t>
+  </si>
+  <si>
     <t>GWL_Item_FP_Pl_Dissimilar_02</t>
+  </si>
+  <si>
+    <t>25405.38</t>
   </si>
   <si>
     <t>GWL_Item_FP_Pl_Dissimilar_03</t>
   </si>
   <si>
-    <t>129.9</t>
+    <t>13258.08</t>
+  </si>
+  <si>
+    <t>205.323</t>
+  </si>
+  <si>
+    <t>14164.93776</t>
+  </si>
+  <si>
+    <t>383.326</t>
+  </si>
+  <si>
+    <t>10044.56288</t>
+  </si>
+  <si>
+    <t>375.327</t>
+  </si>
+  <si>
+    <t>9091.00385</t>
+  </si>
+  <si>
+    <t>14250.20994</t>
+  </si>
+  <si>
+    <t>386.326</t>
+  </si>
+  <si>
+    <t>10129.17345</t>
+  </si>
+  <si>
+    <t>379.327</t>
+  </si>
+  <si>
+    <t>9111.57406</t>
+  </si>
+  <si>
+    <t>14335.06883</t>
+  </si>
+  <si>
+    <t>10212.48006</t>
+  </si>
+  <si>
+    <t>9131.71497</t>
+  </si>
+  <si>
+    <t>206.323</t>
+  </si>
+  <si>
+    <t>14419.51643</t>
+  </si>
+  <si>
+    <t>389.326</t>
+  </si>
+  <si>
+    <t>10295.14474</t>
+  </si>
+  <si>
+    <t>383.327</t>
+  </si>
+  <si>
+    <t>9151.64571</t>
+  </si>
+  <si>
+    <t>207.323</t>
+  </si>
+  <si>
+    <t>14503.14938</t>
+  </si>
+  <si>
+    <t>392.326</t>
+  </si>
+  <si>
+    <t>10376.5452</t>
+  </si>
+  <si>
+    <t>387.327</t>
+  </si>
+  <si>
+    <t>9171.16479</t>
+  </si>
+  <si>
+    <t>235.654</t>
+  </si>
+  <si>
+    <t>12986.52483</t>
+  </si>
+  <si>
+    <t>381.652</t>
+  </si>
+  <si>
+    <t>12015.33048</t>
+  </si>
+  <si>
+    <t>281.327</t>
+  </si>
+  <si>
+    <t>9420.99171</t>
   </si>
 </sst>
 </file>
@@ -1556,7 +1658,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2205,18 +2307,18 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="44" max="44" width="10.1428571428571"/>
     <col min="48" max="48" width="11.7142857142857"/>
-    <col min="50" max="50" width="16.7142857142857" customWidth="1"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="50" max="50" customWidth="true" width="16.7142857142857"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -2615,14 +2717,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f>F4*G4</f>
         <v>750</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -2760,10 +2862,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>82</v>
       </c>
       <c r="AW4" s="25">
@@ -2804,10 +2906,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -2841,14 +2943,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f>F5*G5</f>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -2986,10 +3088,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>94</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>95</v>
       </c>
       <c r="AW5" s="25">
@@ -3030,10 +3132,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -3067,14 +3169,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f>F6*G6</f>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -3212,10 +3314,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>102</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>103</v>
       </c>
       <c r="AW6" s="25">
@@ -3256,10 +3358,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -4441,11 +4543,11 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="27.1428571428571" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="27.1428571428571"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -4844,14 +4946,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>750</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -4989,10 +5091,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -5033,10 +5135,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -5070,14 +5172,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -5215,10 +5317,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -5259,10 +5361,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -5296,14 +5398,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -5441,10 +5543,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -5485,10 +5587,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -6670,14 +6772,14 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
     <col min="52" max="52" width="13.2857142857143"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7076,14 +7178,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>150</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -7221,10 +7323,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>174</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>175</v>
       </c>
       <c r="AW4" s="25">
@@ -7265,10 +7367,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -7302,14 +7404,14 @@
       <c r="F5" s="20">
         <v>6</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>177</v>
       </c>
       <c r="J5" s="20">
@@ -7447,10 +7549,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>178</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>179</v>
       </c>
       <c r="AW5" s="25">
@@ -7491,10 +7593,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -7528,14 +7630,14 @@
       <c r="F6" s="20">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1800</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>181</v>
       </c>
       <c r="J6" s="20">
@@ -7673,10 +7775,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>182</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>183</v>
       </c>
       <c r="AW6" s="25">
@@ -7717,10 +7819,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -8902,16 +9004,16 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.57142857142857"/>
     <col min="35" max="35" width="11.4285714285714"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -9310,14 +9412,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -9455,10 +9557,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>88</v>
       </c>
       <c r="AW4" s="25">
@@ -9499,10 +9601,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -9536,14 +9638,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -9681,10 +9783,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>96</v>
       </c>
       <c r="AW5" s="25">
@@ -9725,10 +9827,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -9762,14 +9864,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -9907,10 +10009,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>104</v>
       </c>
       <c r="AW6" s="25">
@@ -9951,10 +10053,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -11136,15 +11238,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11543,14 +11645,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -11688,11 +11790,11 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
-        <v>188</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>189</v>
+      <c r="AU4" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>259</v>
       </c>
       <c r="AW4" s="25">
         <f t="shared" ref="AW4:AW6" si="12">AM4</f>
@@ -11732,10 +11834,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -11769,14 +11871,14 @@
       <c r="F5" s="20">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -11914,11 +12016,11 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
-        <v>191</v>
-      </c>
-      <c r="AV5" t="s">
-        <v>192</v>
+      <c r="AU5" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="AV5" t="s" s="0">
+        <v>261</v>
       </c>
       <c r="AW5" s="25">
         <f t="shared" si="12"/>
@@ -11958,10 +12060,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -11995,14 +12097,14 @@
       <c r="F6" s="20">
         <v>9</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -12140,11 +12242,11 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
-        <v>194</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>195</v>
+      <c r="AU6" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="AV6" t="s" s="0">
+        <v>263</v>
       </c>
       <c r="AW6" s="25">
         <f t="shared" si="12"/>
@@ -12184,10 +12286,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -13369,14 +13471,14 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="30.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="35" max="35" width="11.4285714285714"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -13775,14 +13877,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -13920,10 +14022,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>197</v>
       </c>
       <c r="AW4" s="25">
@@ -13964,10 +14066,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -14001,14 +14103,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -14146,10 +14248,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>199</v>
       </c>
       <c r="AW5" s="25">
@@ -14190,10 +14292,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -14227,14 +14329,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -14372,10 +14474,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>201</v>
       </c>
       <c r="AW6" s="25">
@@ -14416,10 +14518,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -15601,15 +15703,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="52" max="52" width="13.2857142857143"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -16008,14 +16110,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -16153,10 +16255,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>203</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>204</v>
       </c>
       <c r="AW4" s="25">
@@ -16197,10 +16299,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -16234,14 +16336,14 @@
       <c r="F5" s="20">
         <v>6</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -16379,10 +16481,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>206</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>207</v>
       </c>
       <c r="AW5" s="25">
@@ -16423,10 +16525,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -16460,14 +16562,14 @@
       <c r="F6" s="20">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -16605,10 +16707,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>209</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>210</v>
       </c>
       <c r="AW6" s="25">
@@ -16649,10 +16751,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -17834,14 +17936,14 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="52" max="52" width="13.1428571428571"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -18240,14 +18342,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -18385,10 +18487,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>212</v>
       </c>
       <c r="AW4" s="25">
@@ -18429,10 +18531,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -18466,14 +18568,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -18611,10 +18713,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>214</v>
       </c>
       <c r="AW5" s="25">
@@ -18655,10 +18757,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -18692,14 +18794,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -18837,10 +18939,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>216</v>
       </c>
       <c r="AW6" s="25">
@@ -18881,10 +18983,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -20066,15 +20168,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -20473,14 +20575,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -20618,11 +20720,11 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
-        <v>218</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>219</v>
+      <c r="AU4" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>253</v>
       </c>
       <c r="AW4" s="25">
         <f t="shared" ref="AW4:AW6" si="12">AM4</f>
@@ -20662,10 +20764,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -20699,14 +20801,14 @@
       <c r="F5" s="20">
         <v>9</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -20844,11 +20946,11 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
-        <v>221</v>
-      </c>
-      <c r="AV5" t="s">
-        <v>222</v>
+      <c r="AU5" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="AV5" t="s" s="0">
+        <v>255</v>
       </c>
       <c r="AW5" s="25">
         <f t="shared" si="12"/>
@@ -20888,10 +20990,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -20925,14 +21027,14 @@
       <c r="F6" s="20">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -21070,11 +21172,11 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
-        <v>224</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>225</v>
+      <c r="AU6" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="AV6" t="s" s="0">
+        <v>257</v>
       </c>
       <c r="AW6" s="25">
         <f t="shared" si="12"/>
@@ -21114,10 +21216,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -22299,15 +22401,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="29.447619047619" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="29.447619047619"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="35" max="35" width="11.4285714285714"/>
-    <col min="50" max="50" width="16.7142857142857" customWidth="1"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="50" max="50" customWidth="true" width="16.7142857142857"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -22687,7 +22789,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="19">
         <v>1</v>
       </c>
@@ -22706,14 +22808,14 @@
       <c r="F4" s="20">
         <v>9</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -22851,11 +22953,11 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
-        <v>143</v>
+      <c r="AV4" t="s" s="0">
+        <v>227</v>
       </c>
       <c r="AW4" s="25">
         <f t="shared" ref="AW4:AW6" si="12">AM4</f>
@@ -22895,10 +22997,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -22913,15 +23015,15 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="19">
         <v>1</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>77</v>
@@ -22932,14 +23034,14 @@
       <c r="F5" s="20">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J5" s="20">
@@ -23077,11 +23179,11 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
-        <v>145</v>
+      <c r="AV5" t="s" s="0">
+        <v>229</v>
       </c>
       <c r="AW5" s="25">
         <f t="shared" si="12"/>
@@ -23121,10 +23223,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -23139,15 +23241,15 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="6" spans="1:69">
+    <row r="6" ht="15.75" spans="1:69">
       <c r="A6" s="19">
         <v>1</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>77</v>
@@ -23158,14 +23260,14 @@
       <c r="F6" s="20">
         <v>15</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>750</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J6" s="20">
@@ -23303,11 +23405,11 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV6" t="s">
-        <v>229</v>
+      <c r="AV6" t="s" s="0">
+        <v>231</v>
       </c>
       <c r="AW6" s="25">
         <f t="shared" si="12"/>
@@ -23347,10 +23449,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -24532,15 +24634,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="3" width="32.1428571428571" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="3" customWidth="true" width="32.1428571428571"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="51" max="51" width="14.5714285714286" customWidth="1"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="51" max="51" customWidth="true" width="14.5714285714286"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -24939,14 +25041,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -25084,10 +25186,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>128</v>
       </c>
       <c r="AW4" s="25">
@@ -25128,10 +25230,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -25165,14 +25267,14 @@
       <c r="F5" s="20">
         <v>9</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -25310,10 +25412,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>130</v>
       </c>
       <c r="AW5" s="25">
@@ -25354,10 +25456,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -25391,14 +25493,14 @@
       <c r="F6" s="20">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -25536,10 +25638,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>132</v>
       </c>
       <c r="AW6" s="25">
@@ -25580,10 +25682,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -26765,15 +26867,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="10.5714285714286"/>
     <col min="35" max="35" width="12.8571428571429"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -27172,14 +27274,14 @@
       <c r="F4" s="20">
         <v>12</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>1800</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -27317,10 +27419,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>134</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>135</v>
       </c>
       <c r="AW4" s="25">
@@ -27361,10 +27463,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -27398,14 +27500,14 @@
       <c r="F5" s="20">
         <v>3</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -27543,10 +27645,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>137</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>138</v>
       </c>
       <c r="AW5" s="25">
@@ -27587,10 +27689,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -27624,14 +27726,14 @@
       <c r="F6" s="20">
         <v>9</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -27769,10 +27871,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>140</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>141</v>
       </c>
       <c r="AW6" s="25">
@@ -27813,10 +27915,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -28998,10 +29100,10 @@
   <dimension ref="A1:BQ19"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="18" max="19" width="9.28571428571429"/>
     <col min="20" max="20" width="10.7142857142857"/>
     <col min="29" max="29" width="9.28571428571429"/>
@@ -29011,9 +29113,9 @@
     <col min="49" max="49" width="14.5714285714286"/>
     <col min="50" max="50" width="10.1428571428571"/>
     <col min="51" max="51" width="14.5714285714286"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -29412,14 +29514,14 @@
       <c r="F4" s="20">
         <v>9</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f>F4*G4</f>
         <v>1350</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -29456,7 +29558,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>229.1</v>
       </c>
-      <c r="S4" s="21">
+      <c r="S4" s="20">
         <f>(H4-R4)</f>
         <v>1120.9</v>
       </c>
@@ -29557,10 +29659,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW4" s="25">
@@ -29601,10 +29703,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -29638,14 +29740,14 @@
       <c r="F5" s="20">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f>F5*G5</f>
         <v>1200</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -29783,10 +29885,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>145</v>
       </c>
       <c r="AW5" s="25">
@@ -29827,10 +29929,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -31011,15 +31113,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="52" max="52" width="13.2857142857143"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -31418,14 +31520,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -31563,10 +31665,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -31607,10 +31709,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -31644,14 +31746,14 @@
       <c r="F5" s="20">
         <v>6</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -31789,10 +31891,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -31833,10 +31935,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -31870,14 +31972,14 @@
       <c r="F6" s="20">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -32015,10 +32117,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -32059,10 +32161,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -33244,11 +33346,11 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -33647,14 +33749,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>750</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -33792,10 +33894,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -33836,10 +33938,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -33873,14 +33975,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -34018,10 +34120,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -34062,10 +34164,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -34099,14 +34201,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -34244,10 +34346,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -34288,10 +34390,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -35473,11 +35575,11 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="29.1428571428571" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="29.1428571428571"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -35876,14 +35978,14 @@
       <c r="F4" s="20">
         <v>5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -36021,10 +36123,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -36065,10 +36167,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -36102,14 +36204,14 @@
       <c r="F5" s="20">
         <v>4</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -36247,10 +36349,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -36291,10 +36393,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -36328,14 +36430,14 @@
       <c r="F6" s="20">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -36473,10 +36575,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -36517,10 +36619,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -37702,15 +37804,15 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="29" max="29" width="9.28571428571429"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="52" max="52" width="13.2857142857143"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -38109,14 +38211,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>78</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>450</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>79</v>
       </c>
       <c r="J4" s="20">
@@ -38254,10 +38356,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -38298,10 +38400,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -38335,14 +38437,14 @@
       <c r="F5" s="20">
         <v>6</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -38480,10 +38582,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -38524,10 +38626,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -38561,14 +38663,14 @@
       <c r="F6" s="20">
         <v>9</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -38706,10 +38808,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -38750,10 +38852,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">
@@ -39935,14 +40037,14 @@
   <dimension ref="A1:BQ20"/>
   <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" customWidth="1"/>
-    <col min="14" max="14" width="13.847619047619" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="28.0"/>
+    <col min="3" max="3" customWidth="true" width="23.0"/>
+    <col min="13" max="13" customWidth="true" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" width="13.847619047619"/>
     <col min="35" max="35" width="11.4285714285714"/>
     <col min="52" max="52" width="13.2857142857143"/>
-    <col min="64" max="64" width="11" customWidth="1"/>
-    <col min="67" max="67" width="12"/>
+    <col min="64" max="64" customWidth="true" width="11.0"/>
+    <col min="67" max="67" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -40341,14 +40443,14 @@
       <c r="F4" s="20">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ref="H4:H6" si="0">F4*G4</f>
         <v>150</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J4" s="20">
@@ -40486,10 +40588,10 @@
       <c r="AT4" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" t="s" s="0">
         <v>148</v>
       </c>
       <c r="AW4" s="25">
@@ -40530,10 +40632,10 @@
       <c r="BL4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="BO4" s="25">
@@ -40567,14 +40669,14 @@
       <c r="F5" s="20">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>92</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" t="s" s="0">
         <v>93</v>
       </c>
       <c r="J5" s="20">
@@ -40712,10 +40814,10 @@
       <c r="AT5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" t="s" s="0">
         <v>151</v>
       </c>
       <c r="AW5" s="25">
@@ -40756,10 +40858,10 @@
       <c r="BL5" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM5" t="s">
+      <c r="BM5" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BN5" t="s" s="0">
         <v>97</v>
       </c>
       <c r="BO5" s="25">
@@ -40793,14 +40895,14 @@
       <c r="F6" s="20">
         <v>9</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>100</v>
       </c>
       <c r="H6" s="20">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" t="s" s="0">
         <v>101</v>
       </c>
       <c r="J6" s="20">
@@ -40938,10 +41040,10 @@
       <c r="AT6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AU6" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AV6" t="s" s="0">
         <v>154</v>
       </c>
       <c r="AW6" s="25">
@@ -40982,10 +41084,10 @@
       <c r="BL6" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="BM6" t="s">
+      <c r="BM6" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BN6" t="s">
+      <c r="BN6" t="s" s="0">
         <v>105</v>
       </c>
       <c r="BO6" s="25">

</xml_diff>